<commit_message>
revisi report dan log dan filter
</commit_message>
<xml_diff>
--- a/public/templates/dryer-report-template.xlsx
+++ b/public/templates/dryer-report-template.xlsx
@@ -201,6 +201,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -213,7 +214,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -531,33 +531,33 @@
   <dimension ref="B2:L51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
     <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" customWidth="1"/>
     <col min="7" max="7" width="9.7109375" customWidth="1"/>
     <col min="8" max="8" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:12" ht="14.45" x14ac:dyDescent="0.35">
-      <c r="C2" s="9"/>
-      <c r="J2" s="9"/>
+      <c r="C2" s="5"/>
+      <c r="J2" s="5"/>
     </row>
     <row r="4" spans="2:12" ht="23.45" x14ac:dyDescent="0.55000000000000004">
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
@@ -656,35 +656,35 @@
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="6" t="s">
+      <c r="F10" s="6"/>
+      <c r="G10" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="6"/>
-      <c r="I10" s="5" t="s">
+      <c r="H10" s="7"/>
+      <c r="I10" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="J10" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="K10" s="5"/>
+      <c r="K10" s="6"/>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
       <c r="E11" s="3" t="s">
         <v>17</v>
       </c>
@@ -697,9 +697,9 @@
       <c r="H11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
     </row>
     <row r="12" spans="2:12" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B12" s="1"/>
@@ -710,8 +710,8 @@
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="1"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
     </row>
     <row r="13" spans="2:12" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B13" s="1"/>
@@ -722,8 +722,8 @@
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="1"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
     </row>
     <row r="14" spans="2:12" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B14" s="1"/>
@@ -734,8 +734,8 @@
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
     </row>
     <row r="15" spans="2:12" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B15" s="1"/>
@@ -746,8 +746,8 @@
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="1"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
     </row>
     <row r="16" spans="2:12" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B16" s="1"/>
@@ -758,8 +758,8 @@
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
     </row>
     <row r="17" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -770,8 +770,8 @@
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
     </row>
     <row r="18" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B18" s="1"/>
@@ -782,8 +782,8 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
     </row>
     <row r="19" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B19" s="1"/>
@@ -794,8 +794,8 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="7"/>
-      <c r="K19" s="7"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
     </row>
     <row r="20" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B20" s="1"/>
@@ -806,8 +806,8 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
-      <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
     </row>
     <row r="21" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B21" s="1"/>
@@ -818,8 +818,8 @@
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
     </row>
     <row r="22" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B22" s="1"/>
@@ -830,8 +830,8 @@
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
     </row>
     <row r="23" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B23" s="1"/>
@@ -842,8 +842,8 @@
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
     </row>
     <row r="24" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B24" s="1"/>
@@ -854,8 +854,8 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
     </row>
     <row r="25" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B25" s="1"/>
@@ -866,8 +866,8 @@
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
     </row>
     <row r="26" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
       <c r="B26" s="1"/>
@@ -878,10 +878,10 @@
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-    </row>
-    <row r="27" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -890,10 +890,10 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
-      <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
-    </row>
-    <row r="28" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
@@ -902,10 +902,10 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
-    </row>
-    <row r="29" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+    </row>
+    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
@@ -914,10 +914,10 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
-      <c r="J29" s="7"/>
-      <c r="K29" s="7"/>
-    </row>
-    <row r="30" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+    </row>
+    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
@@ -926,10 +926,10 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
-      <c r="J30" s="7"/>
-      <c r="K30" s="7"/>
-    </row>
-    <row r="31" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+    </row>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -938,10 +938,10 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-    </row>
-    <row r="32" spans="2:11" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+    </row>
+    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -950,8 +950,8 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
-      <c r="J32" s="7"/>
-      <c r="K32" s="7"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B33" s="1"/>
@@ -962,8 +962,8 @@
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
-      <c r="J33" s="7"/>
-      <c r="K33" s="7"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B34" s="1"/>
@@ -974,8 +974,8 @@
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
-      <c r="J34" s="7"/>
-      <c r="K34" s="7"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B35" s="1"/>
@@ -986,8 +986,8 @@
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
-      <c r="J35" s="7"/>
-      <c r="K35" s="7"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
@@ -998,8 +998,8 @@
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
-      <c r="J36" s="7"/>
-      <c r="K36" s="7"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B37" s="1"/>
@@ -1010,8 +1010,8 @@
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
     </row>
     <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B38" s="1"/>
@@ -1022,8 +1022,8 @@
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
-      <c r="J38" s="7"/>
-      <c r="K38" s="7"/>
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
     </row>
     <row r="39" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B39" s="1"/>
@@ -1034,8 +1034,8 @@
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
-      <c r="J39" s="7"/>
-      <c r="K39" s="7"/>
+      <c r="J39" s="8"/>
+      <c r="K39" s="8"/>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
@@ -1046,8 +1046,8 @@
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
-      <c r="J40" s="7"/>
-      <c r="K40" s="7"/>
+      <c r="J40" s="8"/>
+      <c r="K40" s="8"/>
     </row>
     <row r="41" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B41" s="1"/>
@@ -1058,8 +1058,8 @@
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
-      <c r="J41" s="7"/>
-      <c r="K41" s="7"/>
+      <c r="J41" s="8"/>
+      <c r="K41" s="8"/>
     </row>
     <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
@@ -1070,8 +1070,8 @@
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
-      <c r="J42" s="7"/>
-      <c r="K42" s="7"/>
+      <c r="J42" s="8"/>
+      <c r="K42" s="8"/>
     </row>
     <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" s="1"/>
@@ -1082,8 +1082,8 @@
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
-      <c r="J43" s="7"/>
-      <c r="K43" s="7"/>
+      <c r="J43" s="8"/>
+      <c r="K43" s="8"/>
     </row>
     <row r="44" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B44" s="1"/>
@@ -1094,8 +1094,8 @@
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
-      <c r="J44" s="7"/>
-      <c r="K44" s="7"/>
+      <c r="J44" s="8"/>
+      <c r="K44" s="8"/>
     </row>
     <row r="45" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B45" s="1"/>
@@ -1106,8 +1106,8 @@
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
-      <c r="J45" s="7"/>
-      <c r="K45" s="7"/>
+      <c r="J45" s="8"/>
+      <c r="K45" s="8"/>
     </row>
     <row r="46" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B46" s="1"/>
@@ -1118,8 +1118,8 @@
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
-      <c r="J46" s="7"/>
-      <c r="K46" s="7"/>
+      <c r="J46" s="8"/>
+      <c r="K46" s="8"/>
     </row>
     <row r="47" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B47" s="1"/>
@@ -1130,8 +1130,8 @@
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
-      <c r="J47" s="7"/>
-      <c r="K47" s="7"/>
+      <c r="J47" s="8"/>
+      <c r="K47" s="8"/>
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
@@ -1142,8 +1142,8 @@
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
-      <c r="J48" s="7"/>
-      <c r="K48" s="7"/>
+      <c r="J48" s="8"/>
+      <c r="K48" s="8"/>
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
@@ -1154,8 +1154,8 @@
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
-      <c r="J49" s="7"/>
-      <c r="K49" s="7"/>
+      <c r="J49" s="8"/>
+      <c r="K49" s="8"/>
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
@@ -1166,8 +1166,8 @@
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
-      <c r="J50" s="7"/>
-      <c r="K50" s="7"/>
+      <c r="J50" s="8"/>
+      <c r="K50" s="8"/>
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
@@ -1178,8 +1178,8 @@
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
-      <c r="J51" s="7"/>
-      <c r="K51" s="7"/>
+      <c r="J51" s="8"/>
+      <c r="K51" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="48">

</xml_diff>